<commit_message>
changed xlsx file content
</commit_message>
<xml_diff>
--- a/peri peri asins.xlsx
+++ b/peri peri asins.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Mukul ML\Projects\RAG-Langraph-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34DC5596-983E-4943-AD64-EEC32EF442E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2AE607-C720-459E-A458-4DB71C1D0AA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" xr2:uid="{8460192D-109B-4B2F-88EB-CFF0DB0F1D19}"/>
   </bookViews>
@@ -25,45 +25,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="3">
   <si>
     <t>asin</t>
   </si>
   <si>
-    <t>B0G94DXQ4T</t>
+    <t>abcd</t>
   </si>
   <si>
-    <t>B0G94KLCZL</t>
-  </si>
-  <si>
-    <t>B0G94J7NWD</t>
-  </si>
-  <si>
-    <t>B0G94HD8NT</t>
-  </si>
-  <si>
-    <t>B0G71B2K72</t>
-  </si>
-  <si>
-    <t>B0G71LQNP5</t>
-  </si>
-  <si>
-    <t>B0G71SKK72</t>
-  </si>
-  <si>
-    <t>B0G7197ZDK</t>
-  </si>
-  <si>
-    <t>B0G5PTZ8JR</t>
-  </si>
-  <si>
-    <t>B0G5F8835S</t>
-  </si>
-  <si>
-    <t>B0G6L81GQB</t>
-  </si>
-  <si>
-    <t>B0G6LHL8PZ</t>
+    <t>effg</t>
   </si>
 </sst>
 </file>
@@ -437,58 +407,40 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
+      <c r="A5" s="1"/>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="A6" s="1"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
+      <c r="A7" s="1"/>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="A8" s="1"/>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="A9" s="1"/>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>9</v>
-      </c>
+      <c r="A10" s="1"/>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="A11" s="1"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="A12" s="1"/>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="A13" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>